<commit_message>
Updates done up to 7/24/26.
</commit_message>
<xml_diff>
--- a/Results/rbf_fd_parameter_study_2.xlsx
+++ b/Results/rbf_fd_parameter_study_2.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2009,6 +2009,760 @@
         </is>
       </c>
       <c r="Q27" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I28" t="b">
+        <v>0</v>
+      </c>
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.0002757210506970761</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.0001880308200762655</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.0004459234516276548</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.0007564967435892246</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.0009986075880267396</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>30</v>
+      </c>
+      <c r="B29" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I29" t="b">
+        <v>0</v>
+      </c>
+      <c r="J29" t="b">
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>8.94130514132968e-05</v>
+      </c>
+      <c r="L29" t="n">
+        <v>7.653449593435425e-05</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.0002141802374216122</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.0003458890866205636</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.00048285207708024</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>50</v>
+      </c>
+      <c r="B30" t="n">
+        <v>50</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I30" t="b">
+        <v>0</v>
+      </c>
+      <c r="J30" t="b">
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>3.314268206906132e-05</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2.922319519180245e-05</v>
+      </c>
+      <c r="M30" t="n">
+        <v>8.209189593442916e-05</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.0001308872308602571</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.00018349829092921</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>75</v>
+      </c>
+      <c r="B31" t="n">
+        <v>75</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I31" t="b">
+        <v>0</v>
+      </c>
+      <c r="J31" t="b">
+        <v>1</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1.567137032342412e-05</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1.348433417019511e-05</v>
+      </c>
+      <c r="M31" t="n">
+        <v>3.746133250560605e-05</v>
+      </c>
+      <c r="N31" t="n">
+        <v>5.96816038439556e-05</v>
+      </c>
+      <c r="O31" t="n">
+        <v>8.338513803158042e-05</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>100</v>
+      </c>
+      <c r="B32" t="n">
+        <v>100</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J32" t="b">
+        <v>1</v>
+      </c>
+      <c r="K32" t="n">
+        <v>9.016506052198623e-06</v>
+      </c>
+      <c r="L32" t="n">
+        <v>7.711802166165057e-06</v>
+      </c>
+      <c r="M32" t="n">
+        <v>2.131472441604473e-05</v>
+      </c>
+      <c r="N32" t="n">
+        <v>3.400878178126714e-05</v>
+      </c>
+      <c r="O32" t="n">
+        <v>4.736683263658282e-05</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>125</v>
+      </c>
+      <c r="B33" t="n">
+        <v>125</v>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I33" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K33" t="n">
+        <v>5.839171051862862e-06</v>
+      </c>
+      <c r="L33" t="n">
+        <v>4.97939486600134e-06</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.372705919210748e-05</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2.187655074521899e-05</v>
+      </c>
+      <c r="O33" t="n">
+        <v>3.048099287508581e-05</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>150</v>
+      </c>
+      <c r="B34" t="n">
+        <v>150</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I34" t="b">
+        <v>0</v>
+      </c>
+      <c r="J34" t="b">
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>4.079716615261009e-06</v>
+      </c>
+      <c r="L34" t="n">
+        <v>3.476502909351208e-06</v>
+      </c>
+      <c r="M34" t="n">
+        <v>9.569975722855855e-06</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1.525571617696953e-05</v>
+      </c>
+      <c r="O34" t="n">
+        <v>2.124086229863885e-05</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>175</v>
+      </c>
+      <c r="B35" t="n">
+        <v>175</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I35" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35" t="b">
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3.011627808107967e-06</v>
+      </c>
+      <c r="L35" t="n">
+        <v>2.563387142191317e-06</v>
+      </c>
+      <c r="M35" t="n">
+        <v>7.049844127937845e-06</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1.123076415080959e-05</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1.56430925351016e-05</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>200</v>
+      </c>
+      <c r="B36" t="n">
+        <v>200</v>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I36" t="b">
+        <v>0</v>
+      </c>
+      <c r="J36" t="b">
+        <v>1</v>
+      </c>
+      <c r="K36" t="n">
+        <v>2.316321522156805e-06</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1.969452262858244e-06</v>
+      </c>
+      <c r="M36" t="n">
+        <v>5.408347539044994e-06</v>
+      </c>
+      <c r="N36" t="n">
+        <v>8.620772287592269e-06</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1.199732063336666e-05</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q36" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>250</v>
+      </c>
+      <c r="B37" t="n">
+        <v>250</v>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I37" t="b">
+        <v>0</v>
+      </c>
+      <c r="J37" t="b">
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1.485364028350213e-06</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1.263083642923515e-06</v>
+      </c>
+      <c r="M37" t="n">
+        <v>3.469708655526867e-06</v>
+      </c>
+      <c r="N37" t="n">
+        <v>5.529870103939049e-06</v>
+      </c>
+      <c r="O37" t="n">
+        <v>7.696213043069555e-06</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q37" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>300</v>
+      </c>
+      <c r="B38" t="n">
+        <v>300</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I38" t="b">
+        <v>0</v>
+      </c>
+      <c r="J38" t="b">
+        <v>1</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1.053469384622325e-06</v>
+      </c>
+      <c r="L38" t="n">
+        <v>8.904466746138147e-07</v>
+      </c>
+      <c r="M38" t="n">
+        <v>2.417146797857224e-06</v>
+      </c>
+      <c r="N38" t="n">
+        <v>3.85481675877871e-06</v>
+      </c>
+      <c r="O38" t="n">
+        <v>5.353295850368089e-06</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q38" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>500</v>
+      </c>
+      <c r="B39" t="n">
+        <v>500</v>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I39" t="b">
+        <v>0</v>
+      </c>
+      <c r="J39" t="b">
+        <v>1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>5.405278515209248e-07</v>
+      </c>
+      <c r="L39" t="n">
+        <v>4.585782831118184e-07</v>
+      </c>
+      <c r="M39" t="n">
+        <v>9.153166916178774e-07</v>
+      </c>
+      <c r="N39" t="n">
+        <v>1.432082796546632e-06</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1.916320927823261e-06</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q39" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>750</v>
+      </c>
+      <c r="B40" t="n">
+        <v>750</v>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I40" t="b">
+        <v>0</v>
+      </c>
+      <c r="J40" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1.617664251642476e-06</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.461228202166996e-06</v>
+      </c>
+      <c r="M40" t="n">
+        <v>1.433405026894542e-06</v>
+      </c>
+      <c r="N40" t="n">
+        <v>1.027322427349149e-06</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.300340969999672e-06</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
         <v>750</v>
       </c>
     </row>
@@ -2023,7 +2777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2983,6 +3737,876 @@
         <v>30</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>500</v>
+      </c>
+      <c r="B17" t="n">
+        <v>500</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.189077298631476</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.160581100802471</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.1605844947355088</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.1913268879476932</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.1913268898834466</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>500</v>
+      </c>
+      <c r="B18" t="n">
+        <v>500</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.00384003804002427</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.003263143141915273</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.003261373352573354</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.003263970689560207</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.003263986328008423</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>500</v>
+      </c>
+      <c r="B19" t="n">
+        <v>500</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.0005987073099629394</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.0005517024852060242</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.000527172771209683</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.0003238776228220043</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.0003977430065033522</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>500</v>
+      </c>
+      <c r="B20" t="n">
+        <v>500</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3.620856622086499e-05</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.282832128427304e-05</v>
+      </c>
+      <c r="M20" t="n">
+        <v>3.20295649205397e-05</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2.235802993687709e-05</v>
+      </c>
+      <c r="O20" t="n">
+        <v>2.814093251340039e-05</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>500</v>
+      </c>
+      <c r="B21" t="n">
+        <v>500</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>7.222129181147043e-06</v>
+      </c>
+      <c r="L21" t="n">
+        <v>6.172274541716154e-06</v>
+      </c>
+      <c r="M21" t="n">
+        <v>7.289915288287353e-06</v>
+      </c>
+      <c r="N21" t="n">
+        <v>8.731223118066459e-06</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1.100465115521682e-05</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>500</v>
+      </c>
+      <c r="B22" t="n">
+        <v>500</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>7.167308709940751e-06</v>
+      </c>
+      <c r="L22" t="n">
+        <v>6.412464804707686e-06</v>
+      </c>
+      <c r="M22" t="n">
+        <v>6.400834121488268e-06</v>
+      </c>
+      <c r="N22" t="n">
+        <v>4.899426851071117e-06</v>
+      </c>
+      <c r="O22" t="n">
+        <v>6.348035241224952e-06</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>500</v>
+      </c>
+      <c r="B23" t="n">
+        <v>500</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5.405278515209248e-07</v>
+      </c>
+      <c r="L23" t="n">
+        <v>4.585782831118184e-07</v>
+      </c>
+      <c r="M23" t="n">
+        <v>9.153166916178774e-07</v>
+      </c>
+      <c r="N23" t="n">
+        <v>1.432082796546632e-06</v>
+      </c>
+      <c r="O23" t="n">
+        <v>1.916320927823261e-06</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>500</v>
+      </c>
+      <c r="B24" t="n">
+        <v>500</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1.641902089292083e-05</v>
+      </c>
+      <c r="L24" t="n">
+        <v>1.476272832775284e-05</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1.457989866150315e-05</v>
+      </c>
+      <c r="N24" t="n">
+        <v>1.076279005845392e-05</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1.372369876824609e-05</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>500</v>
+      </c>
+      <c r="B25" t="n">
+        <v>500</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4.613653546455149e-05</v>
+      </c>
+      <c r="L25" t="n">
+        <v>4.210668610684143e-05</v>
+      </c>
+      <c r="M25" t="n">
+        <v>4.075157505071832e-05</v>
+      </c>
+      <c r="N25" t="n">
+        <v>2.708524441250244e-05</v>
+      </c>
+      <c r="O25" t="n">
+        <v>3.396247415632201e-05</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>500</v>
+      </c>
+      <c r="B26" t="n">
+        <v>500</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.0001657852270685771</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.0001533279243583069</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.0001468463622887232</v>
+      </c>
+      <c r="N26" t="n">
+        <v>8.784721126371284e-05</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.0001130133194943837</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>500</v>
+      </c>
+      <c r="B27" t="n">
+        <v>500</v>
+      </c>
+      <c r="C27" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I27" t="b">
+        <v>0</v>
+      </c>
+      <c r="J27" t="b">
+        <v>1</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.001112179461645204</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.001040999171856886</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.000993452573280729</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.0005364251495776959</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.0007408550578970063</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>500</v>
+      </c>
+      <c r="B28" t="n">
+        <v>500</v>
+      </c>
+      <c r="C28" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I28" t="b">
+        <v>0</v>
+      </c>
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.00384459047541269</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.003599765924040152</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.003435002749569078</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.001844578153132325</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.002552735343720557</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>500</v>
+      </c>
+      <c r="B29" t="n">
+        <v>500</v>
+      </c>
+      <c r="C29" t="n">
+        <v>15</v>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I29" t="b">
+        <v>0</v>
+      </c>
+      <c r="J29" t="b">
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.02108506722891057</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.01963503447649544</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.01874060134943081</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.01038976981330928</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.01373588097101363</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>500</v>
+      </c>
+      <c r="B30" t="n">
+        <v>500</v>
+      </c>
+      <c r="C30" t="n">
+        <v>20</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I30" t="b">
+        <v>0</v>
+      </c>
+      <c r="J30" t="b">
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.07119336478287577</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.06619845522323374</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.0631895639553019</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.03403232083196017</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.04433709741652209</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>500</v>
+      </c>
+      <c r="B31" t="n">
+        <v>500</v>
+      </c>
+      <c r="C31" t="n">
+        <v>30</v>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I31" t="b">
+        <v>0</v>
+      </c>
+      <c r="J31" t="b">
+        <v>1</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.5031842322014282</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.4685473621227775</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.4472056680312433</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.1765833449404199</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.2277424738328437</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Experiments corrected with proper conditioning.
</commit_message>
<xml_diff>
--- a/Results/rbf_fd_parameter_study_2.xlsx
+++ b/Results/rbf_fd_parameter_study_2.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2763,6 +2763,760 @@
         </is>
       </c>
       <c r="Q40" t="n">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>20</v>
+      </c>
+      <c r="B41" t="n">
+        <v>20</v>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I41" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.0002358360788938131</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.0001880308200762655</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.0004459234516276548</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0.0007564967435892246</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.0009986075880267396</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q41" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>30</v>
+      </c>
+      <c r="B42" t="n">
+        <v>30</v>
+      </c>
+      <c r="C42" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I42" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" t="b">
+        <v>1</v>
+      </c>
+      <c r="K42" t="n">
+        <v>7.68543233689248e-05</v>
+      </c>
+      <c r="L42" t="n">
+        <v>7.653449593435425e-05</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.0002141802374216122</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.0003458890866205636</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.00048285207708024</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>50</v>
+      </c>
+      <c r="B43" t="n">
+        <v>50</v>
+      </c>
+      <c r="C43" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I43" t="b">
+        <v>0</v>
+      </c>
+      <c r="J43" t="b">
+        <v>1</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2.822068617853745e-05</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.922319519180245e-05</v>
+      </c>
+      <c r="M43" t="n">
+        <v>8.209189593442916e-05</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.0001308872308602571</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.00018349829092921</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q43" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>75</v>
+      </c>
+      <c r="B44" t="n">
+        <v>75</v>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.3291742567397e-05</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.348433417019511e-05</v>
+      </c>
+      <c r="M44" t="n">
+        <v>3.746133250560605e-05</v>
+      </c>
+      <c r="N44" t="n">
+        <v>5.96816038439556e-05</v>
+      </c>
+      <c r="O44" t="n">
+        <v>8.338513803158042e-05</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q44" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>100</v>
+      </c>
+      <c r="B45" t="n">
+        <v>100</v>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I45" t="b">
+        <v>0</v>
+      </c>
+      <c r="J45" t="b">
+        <v>1</v>
+      </c>
+      <c r="K45" t="n">
+        <v>7.658026210650555e-06</v>
+      </c>
+      <c r="L45" t="n">
+        <v>7.711802166165057e-06</v>
+      </c>
+      <c r="M45" t="n">
+        <v>2.131472441604473e-05</v>
+      </c>
+      <c r="N45" t="n">
+        <v>3.400878178126714e-05</v>
+      </c>
+      <c r="O45" t="n">
+        <v>4.736683263658282e-05</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q45" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>125</v>
+      </c>
+      <c r="B46" t="n">
+        <v>125</v>
+      </c>
+      <c r="C46" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I46" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" t="b">
+        <v>1</v>
+      </c>
+      <c r="K46" t="n">
+        <v>4.956295388826454e-06</v>
+      </c>
+      <c r="L46" t="n">
+        <v>4.97939486600134e-06</v>
+      </c>
+      <c r="M46" t="n">
+        <v>1.372705919210748e-05</v>
+      </c>
+      <c r="N46" t="n">
+        <v>2.187655074521899e-05</v>
+      </c>
+      <c r="O46" t="n">
+        <v>3.048099287508581e-05</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>150</v>
+      </c>
+      <c r="B47" t="n">
+        <v>150</v>
+      </c>
+      <c r="C47" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I47" t="b">
+        <v>0</v>
+      </c>
+      <c r="J47" t="b">
+        <v>1</v>
+      </c>
+      <c r="K47" t="n">
+        <v>3.465682014775633e-06</v>
+      </c>
+      <c r="L47" t="n">
+        <v>3.476502909351208e-06</v>
+      </c>
+      <c r="M47" t="n">
+        <v>9.569975722855855e-06</v>
+      </c>
+      <c r="N47" t="n">
+        <v>1.525571617696953e-05</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.124086229863885e-05</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q47" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>175</v>
+      </c>
+      <c r="B48" t="n">
+        <v>175</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I48" t="b">
+        <v>0</v>
+      </c>
+      <c r="J48" t="b">
+        <v>1</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2.557408806440619e-06</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.563387142191317e-06</v>
+      </c>
+      <c r="M48" t="n">
+        <v>7.049844127937845e-06</v>
+      </c>
+      <c r="N48" t="n">
+        <v>1.123076415080959e-05</v>
+      </c>
+      <c r="O48" t="n">
+        <v>1.56430925351016e-05</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q48" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>200</v>
+      </c>
+      <c r="B49" t="n">
+        <v>200</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I49" t="b">
+        <v>0</v>
+      </c>
+      <c r="J49" t="b">
+        <v>1</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.967676710891083e-06</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.969452262858244e-06</v>
+      </c>
+      <c r="M49" t="n">
+        <v>5.408347539044994e-06</v>
+      </c>
+      <c r="N49" t="n">
+        <v>8.620772287592269e-06</v>
+      </c>
+      <c r="O49" t="n">
+        <v>1.199732063336666e-05</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q49" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>250</v>
+      </c>
+      <c r="B50" t="n">
+        <v>250</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>5</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I50" t="b">
+        <v>0</v>
+      </c>
+      <c r="J50" t="b">
+        <v>1</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1.261715303731978e-06</v>
+      </c>
+      <c r="L50" t="n">
+        <v>1.263083642923515e-06</v>
+      </c>
+      <c r="M50" t="n">
+        <v>3.469708655526867e-06</v>
+      </c>
+      <c r="N50" t="n">
+        <v>5.529870103939049e-06</v>
+      </c>
+      <c r="O50" t="n">
+        <v>7.696213043069555e-06</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q50" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>300</v>
+      </c>
+      <c r="B51" t="n">
+        <v>300</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I51" t="b">
+        <v>0</v>
+      </c>
+      <c r="J51" t="b">
+        <v>1</v>
+      </c>
+      <c r="K51" t="n">
+        <v>8.947931211680768e-07</v>
+      </c>
+      <c r="L51" t="n">
+        <v>8.904466746138147e-07</v>
+      </c>
+      <c r="M51" t="n">
+        <v>2.417146797857224e-06</v>
+      </c>
+      <c r="N51" t="n">
+        <v>3.85481675877871e-06</v>
+      </c>
+      <c r="O51" t="n">
+        <v>5.353295850368089e-06</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q51" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>500</v>
+      </c>
+      <c r="B52" t="n">
+        <v>500</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I52" t="b">
+        <v>0</v>
+      </c>
+      <c r="J52" t="b">
+        <v>1</v>
+      </c>
+      <c r="K52" t="n">
+        <v>4.590735774498112e-07</v>
+      </c>
+      <c r="L52" t="n">
+        <v>4.585782831118184e-07</v>
+      </c>
+      <c r="M52" t="n">
+        <v>9.153166916178774e-07</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1.432082796546632e-06</v>
+      </c>
+      <c r="O52" t="n">
+        <v>1.916320927823261e-06</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>750</v>
+      </c>
+      <c r="B53" t="n">
+        <v>750</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I53" t="b">
+        <v>0</v>
+      </c>
+      <c r="J53" t="b">
+        <v>1</v>
+      </c>
+      <c r="K53" t="n">
+        <v>1.373849350562543e-06</v>
+      </c>
+      <c r="L53" t="n">
+        <v>1.461228202166996e-06</v>
+      </c>
+      <c r="M53" t="n">
+        <v>1.433405026894542e-06</v>
+      </c>
+      <c r="N53" t="n">
+        <v>1.027322427349149e-06</v>
+      </c>
+      <c r="O53" t="n">
+        <v>1.300340969999672e-06</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>N_int</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
         <v>750</v>
       </c>
     </row>
@@ -2777,7 +3531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4607,6 +5361,876 @@
         <v>30</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>500</v>
+      </c>
+      <c r="B32" t="n">
+        <v>500</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I32" t="b">
+        <v>0</v>
+      </c>
+      <c r="J32" t="b">
+        <v>1</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.1605844946806367</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.160581100802471</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.1605844947355088</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.1913268879476932</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.1913268898834466</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>500</v>
+      </c>
+      <c r="B33" t="n">
+        <v>500</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I33" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.00326136756064837</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.003263143141915273</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.003261373352573354</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.003263970689560207</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.003263986328008423</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>500</v>
+      </c>
+      <c r="B34" t="n">
+        <v>500</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I34" t="b">
+        <v>0</v>
+      </c>
+      <c r="J34" t="b">
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.0005084857438088917</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.0005517024852060242</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.000527172771209683</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.0003238776228220043</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.0003977430065033522</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>500</v>
+      </c>
+      <c r="B35" t="n">
+        <v>500</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I35" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35" t="b">
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3.075215455146145e-05</v>
+      </c>
+      <c r="L35" t="n">
+        <v>3.282832128427304e-05</v>
+      </c>
+      <c r="M35" t="n">
+        <v>3.20295649205397e-05</v>
+      </c>
+      <c r="N35" t="n">
+        <v>2.235802993687709e-05</v>
+      </c>
+      <c r="O35" t="n">
+        <v>2.814093251340039e-05</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>500</v>
+      </c>
+      <c r="B36" t="n">
+        <v>500</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I36" t="b">
+        <v>0</v>
+      </c>
+      <c r="J36" t="b">
+        <v>1</v>
+      </c>
+      <c r="K36" t="n">
+        <v>6.133798046973533e-06</v>
+      </c>
+      <c r="L36" t="n">
+        <v>6.172274541716154e-06</v>
+      </c>
+      <c r="M36" t="n">
+        <v>7.289915288287353e-06</v>
+      </c>
+      <c r="N36" t="n">
+        <v>8.731223118066459e-06</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1.100465115521682e-05</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q36" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>500</v>
+      </c>
+      <c r="B37" t="n">
+        <v>500</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I37" t="b">
+        <v>0</v>
+      </c>
+      <c r="J37" t="b">
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
+        <v>6.087238688814016e-06</v>
+      </c>
+      <c r="L37" t="n">
+        <v>6.412464804707686e-06</v>
+      </c>
+      <c r="M37" t="n">
+        <v>6.400834121488268e-06</v>
+      </c>
+      <c r="N37" t="n">
+        <v>4.899426851071117e-06</v>
+      </c>
+      <c r="O37" t="n">
+        <v>6.348035241224952e-06</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q37" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>500</v>
+      </c>
+      <c r="B38" t="n">
+        <v>500</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I38" t="b">
+        <v>0</v>
+      </c>
+      <c r="J38" t="b">
+        <v>1</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4.590735774498112e-07</v>
+      </c>
+      <c r="L38" t="n">
+        <v>4.585782831118184e-07</v>
+      </c>
+      <c r="M38" t="n">
+        <v>9.153166916178774e-07</v>
+      </c>
+      <c r="N38" t="n">
+        <v>1.432082796546632e-06</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1.916320927823261e-06</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q38" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>500</v>
+      </c>
+      <c r="B39" t="n">
+        <v>500</v>
+      </c>
+      <c r="C39" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I39" t="b">
+        <v>0</v>
+      </c>
+      <c r="J39" t="b">
+        <v>1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1.394477386933422e-05</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1.476272832775284e-05</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1.457989866150315e-05</v>
+      </c>
+      <c r="N39" t="n">
+        <v>1.076279005845392e-05</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1.372369876824609e-05</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q39" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>500</v>
+      </c>
+      <c r="B40" t="n">
+        <v>500</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I40" t="b">
+        <v>0</v>
+      </c>
+      <c r="J40" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" t="n">
+        <v>3.918403894869758e-05</v>
+      </c>
+      <c r="L40" t="n">
+        <v>4.210668610684143e-05</v>
+      </c>
+      <c r="M40" t="n">
+        <v>4.075157505071832e-05</v>
+      </c>
+      <c r="N40" t="n">
+        <v>2.708524441250244e-05</v>
+      </c>
+      <c r="O40" t="n">
+        <v>3.396247415632201e-05</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>500</v>
+      </c>
+      <c r="B41" t="n">
+        <v>500</v>
+      </c>
+      <c r="C41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I41" t="b">
+        <v>0</v>
+      </c>
+      <c r="J41" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.0001408023972577012</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.0001533279243583069</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.0001468463622887232</v>
+      </c>
+      <c r="N41" t="n">
+        <v>8.784721126371284e-05</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.0001130133194943837</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q41" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>500</v>
+      </c>
+      <c r="B42" t="n">
+        <v>500</v>
+      </c>
+      <c r="C42" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I42" t="b">
+        <v>0</v>
+      </c>
+      <c r="J42" t="b">
+        <v>1</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.0009445807515506046</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.001040999171856886</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.000993452573280729</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.0005364251495776959</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.0007408550578970063</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>500</v>
+      </c>
+      <c r="B43" t="n">
+        <v>500</v>
+      </c>
+      <c r="C43" t="n">
+        <v>10</v>
+      </c>
+      <c r="D43" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I43" t="b">
+        <v>0</v>
+      </c>
+      <c r="J43" t="b">
+        <v>1</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.003265233971590916</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.003599765924040152</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.003435002749569078</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.001844578153132325</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.002552735343720557</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q43" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>500</v>
+      </c>
+      <c r="B44" t="n">
+        <v>500</v>
+      </c>
+      <c r="C44" t="n">
+        <v>15</v>
+      </c>
+      <c r="D44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.01790767527761895</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.01963503447649544</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.01874060134943081</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0.01038976981330928</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.01373588097101363</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q44" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>500</v>
+      </c>
+      <c r="B45" t="n">
+        <v>500</v>
+      </c>
+      <c r="C45" t="n">
+        <v>20</v>
+      </c>
+      <c r="D45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I45" t="b">
+        <v>0</v>
+      </c>
+      <c r="J45" t="b">
+        <v>1</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.06046495581976309</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.06619845522323374</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.0631895639553019</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0.03403232083196017</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.04433709741652209</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q45" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>500</v>
+      </c>
+      <c r="B46" t="n">
+        <v>500</v>
+      </c>
+      <c r="C46" t="n">
+        <v>30</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>lambda p: 1e0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>lambda p: 1e-3</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>lambda p: 12.0/24.0*np.pi</t>
+        </is>
+      </c>
+      <c r="I46" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" t="b">
+        <v>1</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.4273574154283958</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.4685473621227775</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.4472056680312433</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0.1765833449404199</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.2277424738328437</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Inverse Length Scale</t>
+        </is>
+      </c>
+      <c r="Q46" t="n">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>